<commit_message>
test: 21 tests ajoutés — corrections mockup (P-087→P-096) + consortium FR59 (P-097→P-107)
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/tests_module_projet.xlsx
+++ b/backend/tests_module_projet.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2360,6 +2360,811 @@
       <c r="H58" s="4" t="inlineStr"/>
       <c r="I58" s="3" t="inlineStr"/>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Corrections Mockup</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>P-087</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Wizard - Public/Privé (E-12)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Cocher/décocher Public</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Wizard étape 1</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>1. Ouvrir wizard
+2. Décocher "Projet public"</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Champ is_public=false enregistré, badge "Privé" sur fiche</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>P-088</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Wizard - Consortium (E-13)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Activer consortium + sélection</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Consortium existant</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>1. Cocher "Consortium"
+2. Sélectionner un consortium dans dropdown</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Projet créé avec consortium FK, affiché dans Vue d'ensemble</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>P-089</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Wizard - Services transversaux (E-14)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Sélectionner services</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Wizard étape 1</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>1. Cliquer sur BIM, DD, Paysage
+2. Créer le projet</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Services enregistrés et affichés dans Vue d'ensemble</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>P-090</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Wizard - Créer client (E-15)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Lien créer nouveau client</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Wizard étape 1</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>1. Cliquer champ Client
+2. Vérifier lien "+ Créer un nouveau client"</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Lien visible en bas du dropdown, redirige vers /clients</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>P-091</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Wizard - Sous-traitants (E-09/10)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Étape 4 Sous-traitants</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Wizard étape 4</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>1. Avancer jusqu'à étape 4
+2. Ajouter un ST (nom, spécialité, montant)
+3. Supprimer le ST</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Formulaire ST fonctionnel, 5 étapes au total</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>P-092</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Template - Phase Qualité (E-23)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Vérifier phase QA dans template</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Template ARCH-STD</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>1. Créer projet avec template ARCH-STD
+2. Vérifier phases</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>7 phases dont "Qualité" (QA) avec 3 tâches</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>P-093</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Fiche - Onglet Temps (E-24)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Affichage feuilles de temps projet</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Projet avec entrées de temps</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>1. Ouvrir fiche projet
+2. Cliquer onglet "Temps"</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Tableau: Employé, Date, Phase, Tâche, Heures, Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>P-094</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Fiche - Vue d'ensemble enrichie (E-26/27)</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>KPIs financiers + tableau phases</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Projet avec phases et budget</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>1. Ouvrir fiche projet
+2. Onglet Vue d'ensemble</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>4 KPIs (Budget, Facturé, Consommé, Solde) + tableau phases</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>P-095</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Liste - Colonnes PM/BU/Santé (E-35)</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Vérifier nouvelles colonnes</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Plusieurs projets</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>1. Ouvrir /projects</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>8 colonnes: Code, Nom, Client, CP, BU, Type, Statut, Santé</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>P-096</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Liste - Filtres dropdown (E-36)</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Filtrer par statut/BU/PM</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Projets avec BU variées</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>1. Sélectionner filtre Statut=Actif
+2. Sélectionner filtre BU
+3. Sélectionner filtre CP</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Liste filtrée correctement pour chaque critère</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Consortium (FR59)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>P-097</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Consortium - Création</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Créer un consortium via API</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Client existant</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>1. POST /api/v1/consortiums/
+2. Nom, client, rôle PR=MANDATAIRE</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Consortium créé avec status=ACTIVE</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>P-098</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Consortium - Ajout membre PR</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Ajouter Provencher Roy comme membre</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Consortium existant</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>1. POST /consortiums/{id}/members/
+2. is_pr=true, coefficient=40%</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Membre créé, display_name="Provencher Roy"</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>P-099</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Consortium - Ajout membre externe</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Ajouter organisation externe</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Consortium + org externe</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>1. POST /consortiums/{id}/members/
+2. organization=ID, coefficient=60%</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Membre créé, organization_name correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>P-100</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Consortium - Validation coefficients</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Vérifier somme = 100%</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Consortium avec 2 membres</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>1. GET /consortiums/{id}/validate_coefficients/</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>total_coefficient=100.00, is_valid=true</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>P-101</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Consortium - Coefficients invalides</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Somme != 100%</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Consortium avec 1 membre</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>1. Ajouter un seul membre à 50%
+2. Valider</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>total_coefficient=50, is_valid=false</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>P-102</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Consortium - Association projet</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Associer projet à consortium</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Consortium existant</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>1. Wizard: cocher Consortium
+2. Sélectionner consortium
+3. Créer projet</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Projet.consortium FK renseigné, is_consortium=true</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>P-103</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Consortium - Affichage fiche projet</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Section consortium dans Vue d'ensemble</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Projet consortium</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>1. Ouvrir fiche projet consortium</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Section consortium: nom, client, rôle PR, membres avec %</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>P-104</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Consortium - Unicité membre</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Même org ne peut être ajoutée 2x</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Consortium avec membre</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>1. Ajouter même organisation une 2e fois</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Erreur 400 ou contrainte d'unicité</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>P-105</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Consortium - Suppression membre</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Retirer un membre</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Consortium avec membres</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>1. DELETE /consortiums/{id}/members/{mid}/</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Membre supprimé, coefficient total mis à jour</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>P-106</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Consortium - Liste</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Lister les consortiums</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>1. GET /api/v1/consortiums/</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Liste avec name, client_name, members_count, total_coefficient</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>P-107</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Consortium - Rôle Partenaire</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Créer consortium en tant que Partenaire</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>FINANCE</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Client existant</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>1. Créer consortium pr_role=PARTENAIRE</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Rôle affiché "Partenaire" dans la fiche</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>